<commit_message>
Close the last two gaps against design section 10.2
* SOURCE_COVERAGE_REPORTED: an absent or empty source must be recorded as
  coverage, never read as "the patient had none". The shape fixture now ships one
  sheet with a header and no rows so the distinction is actually exercised.
* MEDS_LINEAGE_COMPLETE: every published MEDS row names the source rows behind
  it. Canonical and OMOP already had this check; MEDS did not.

validate.py's docstring now maps design section 10.2's thirty requirements to
where each is checked, including the ones that are better expressed as tests —
the measured baselines, determinism across worker counts, resumption after a
crash — so the coverage claim is auditable rather than asserted.
</commit_message>
<xml_diff>
--- a/tests/fixtures/ctpe_shape/batch1/no_finding/b1_no.xlsx
+++ b/tests/fixtures/ctpe_shape/batch1/no_finding/b1_no.xlsx
@@ -749,7 +749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -797,45 +797,6 @@
         <is>
           <t>Closest_to_CT</t>
         </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>SUBJ-3</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>ENC-SUBJ-3-1</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>PULMONARY FUNCTION TEST</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2019-03-04</t>
-        </is>
-      </c>
-      <c r="E2" s="1" t="n">
-        <v>43530.38541666666</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>FEV1 PCT PRED</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H2" t="n">
-        <v>78</v>
-      </c>
-      <c r="I2" t="n">
-        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>